<commit_message>
[UPDATE] Memo Btn Add
</commit_message>
<xml_diff>
--- a/Assets/Resources/Xlsx/AssetAddress.xlsx
+++ b/Assets/Resources/Xlsx/AssetAddress.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\KGA\Documents\ProjectVCG\Assets\Resources\Xlsx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\KGA\Desktop\dev\ProjectVCG\Assets\Resources\Xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="GameObject" sheetId="12" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="120">
   <si>
     <r>
       <t>n</t>
@@ -444,6 +444,13 @@
   </si>
   <si>
     <t>Assets/Resources_Addressable/Prefabs/Items/Object_Food_Tuna.prefab</t>
+  </si>
+  <si>
+    <t>Assets/Resources_Addressable/Materials/Logic/MemoMat.mat</t>
+  </si>
+  <si>
+    <t>MemoMat</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1053,7 +1060,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31.140625" customWidth="1"/>
@@ -1162,6 +1169,14 @@
       </c>
       <c r="B13" s="1" t="s">
         <v>52</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B14" t="s">
+        <v>118</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[Update] SheetManager 수정, InteractableManager수정,  함수 블록의 기능 구현
</commit_message>
<xml_diff>
--- a/Assets/Resources/Xlsx/AssetAddress.xlsx
+++ b/Assets/Resources/Xlsx/AssetAddress.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="138">
   <si>
     <r>
       <t>n</t>
@@ -494,6 +494,27 @@
   </si>
   <si>
     <t>Assets/Resources_Addressable/Prefabs/Items/Prefab_Sushi_Shrimp.prefab</t>
+  </si>
+  <si>
+    <t>FunctionMat</t>
+  </si>
+  <si>
+    <t>Assets/Resources_Addressable/Materials/Logic/FunctionMat.mat</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Assets/Resources_Addressable/Prefabs/WorldUI/Sheet/FunctionSheet.prefab</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>FunctionSheet</t>
+  </si>
+  <si>
+    <t>Assets/Resources_Addressable/Prefabs/BlockLogic/FunctionBlockLogic.prefab</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>FunctionBlockLogic</t>
   </si>
 </sst>
 </file>
@@ -788,7 +809,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B38"/>
+  <dimension ref="A1:B40"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31.140625" customWidth="1"/>
@@ -893,210 +914,226 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>55</v>
+        <v>137</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>58</v>
+        <v>22</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B16" s="5" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A16" s="5" t="s">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B17" s="4" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A17" s="4" t="s">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B18" s="5" t="s">
         <v>57</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A18" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
-        <v>73</v>
+        <v>26</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>74</v>
+        <v>54</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>89</v>
+        <v>74</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B25" s="4" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A25" s="4" t="s">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B26" s="4" t="s">
         <v>85</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A26" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A29" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="B29" s="4" t="s">
         <v>87</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A29" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>125</v>
+        <v>115</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" s="6" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="B32" s="5" t="s">
-        <v>126</v>
+        <v>116</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>127</v>
+        <v>119</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" s="6" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" s="6" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" s="6" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A38" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="B37" s="4" t="s">
+      <c r="B38" s="4" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A38" s="4" t="s">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A39" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="B38" s="4" t="s">
+      <c r="B39" s="4" t="s">
         <v>112</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A40" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -1108,7 +1145,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31.140625" customWidth="1"/>
@@ -1241,6 +1278,14 @@
       </c>
       <c r="B16" t="s">
         <v>105</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>132</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>133</v>
       </c>
     </row>
   </sheetData>

</xml_diff>